<commit_message>
#4 Ic MIMXRT1062DVJ6B price updated in BOM
</commit_message>
<xml_diff>
--- a/Design Files/DC-Motor-Driver/BOM/eSpark BOM.xlsx
+++ b/Design Files/DC-Motor-Driver/BOM/eSpark BOM.xlsx
@@ -1149,9 +1149,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
-    <numFmt numFmtId="166" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
-    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="26">
     <font>
@@ -1667,7 +1667,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1703,13 +1703,13 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="17" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="17" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1718,7 +1718,7 @@
     <xf numFmtId="0" fontId="20" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1766,10 +1766,10 @@
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1789,6 +1789,44 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1821,44 +1859,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2279,15 +2279,15 @@
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="69"/>
-      <c r="R1" s="69"/>
-      <c r="S1" s="70"/>
+      <c r="K1" s="83"/>
+      <c r="L1" s="83"/>
+      <c r="M1" s="83"/>
+      <c r="N1" s="83"/>
+      <c r="O1" s="83"/>
+      <c r="P1" s="83"/>
+      <c r="Q1" s="83"/>
+      <c r="R1" s="83"/>
+      <c r="S1" s="84"/>
     </row>
     <row r="2" spans="1:19" ht="31.5">
       <c r="A2" s="2"/>
@@ -2337,7 +2337,7 @@
       <c r="P3" s="13"/>
       <c r="Q3" s="13"/>
       <c r="R3" s="13"/>
-      <c r="S3" s="73"/>
+      <c r="S3" s="87"/>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="2"/>
@@ -2362,7 +2362,7 @@
       <c r="P4" s="17"/>
       <c r="Q4" s="17"/>
       <c r="R4" s="17"/>
-      <c r="S4" s="74"/>
+      <c r="S4" s="88"/>
     </row>
     <row r="5" spans="1:19">
       <c r="A5" s="2"/>
@@ -2387,7 +2387,7 @@
       <c r="P5" s="17"/>
       <c r="Q5" s="17"/>
       <c r="R5" s="17"/>
-      <c r="S5" s="74"/>
+      <c r="S5" s="88"/>
     </row>
     <row r="6" spans="1:19">
       <c r="A6" s="2"/>
@@ -2408,7 +2408,7 @@
       <c r="P6" s="17"/>
       <c r="Q6" s="17"/>
       <c r="R6" s="17"/>
-      <c r="S6" s="74"/>
+      <c r="S6" s="88"/>
     </row>
     <row r="7" spans="1:19">
       <c r="A7" s="2"/>
@@ -2429,7 +2429,7 @@
       <c r="P7" s="26"/>
       <c r="Q7" s="26"/>
       <c r="R7" s="26"/>
-      <c r="S7" s="74"/>
+      <c r="S7" s="88"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1">
       <c r="A8" s="2"/>
@@ -2450,7 +2450,7 @@
       <c r="P8" s="26"/>
       <c r="Q8" s="26"/>
       <c r="R8" s="26"/>
-      <c r="S8" s="74"/>
+      <c r="S8" s="88"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1">
       <c r="A9" s="2"/>
@@ -5189,11 +5189,11 @@
         <v>316</v>
       </c>
       <c r="P57" s="44">
-        <v>8.3000000000000007</v>
+        <v>16.25</v>
       </c>
       <c r="Q57" s="44">
         <f t="shared" si="2"/>
-        <v>49.800000000000004</v>
+        <v>97.5</v>
       </c>
       <c r="R57" s="37"/>
       <c r="S57" s="37"/>
@@ -5851,17 +5851,17 @@
       <c r="K70" s="56"/>
       <c r="L70" s="56"/>
       <c r="M70" s="56"/>
-      <c r="N70" s="71" t="s">
+      <c r="N70" s="85" t="s">
         <v>359</v>
       </c>
-      <c r="O70" s="72"/>
-      <c r="P70" s="72"/>
+      <c r="O70" s="86"/>
+      <c r="P70" s="86"/>
       <c r="Q70" s="61">
         <f>SUM(Q10:Q69)</f>
-        <v>349.80709999999999</v>
-      </c>
-      <c r="R70" s="75"/>
-      <c r="S70" s="76"/>
+        <v>397.50710000000004</v>
+      </c>
+      <c r="R70" s="89"/>
+      <c r="S70" s="90"/>
     </row>
     <row r="71" spans="1:19" ht="18.75">
       <c r="A71" s="2"/>
@@ -5877,17 +5877,17 @@
       <c r="K71" s="60"/>
       <c r="L71" s="60"/>
       <c r="M71" s="60"/>
-      <c r="N71" s="71" t="s">
+      <c r="N71" s="85" t="s">
         <v>360</v>
       </c>
-      <c r="O71" s="72"/>
-      <c r="P71" s="72"/>
+      <c r="O71" s="86"/>
+      <c r="P71" s="86"/>
       <c r="Q71" s="62">
         <f>Q70/5</f>
-        <v>69.961420000000004</v>
-      </c>
-      <c r="R71" s="77"/>
-      <c r="S71" s="78"/>
+        <v>79.50142000000001</v>
+      </c>
+      <c r="R71" s="91"/>
+      <c r="S71" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -5997,15 +5997,15 @@
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="69"/>
-      <c r="R1" s="69"/>
-      <c r="S1" s="70"/>
+      <c r="K1" s="83"/>
+      <c r="L1" s="83"/>
+      <c r="M1" s="83"/>
+      <c r="N1" s="83"/>
+      <c r="O1" s="83"/>
+      <c r="P1" s="83"/>
+      <c r="Q1" s="83"/>
+      <c r="R1" s="83"/>
+      <c r="S1" s="84"/>
     </row>
     <row r="2" spans="1:19" ht="31.5">
       <c r="A2" s="2"/>
@@ -6055,7 +6055,7 @@
       <c r="P3" s="13"/>
       <c r="Q3" s="13"/>
       <c r="R3" s="13"/>
-      <c r="S3" s="73"/>
+      <c r="S3" s="87"/>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="2"/>
@@ -6080,7 +6080,7 @@
       <c r="P4" s="17"/>
       <c r="Q4" s="17"/>
       <c r="R4" s="17"/>
-      <c r="S4" s="74"/>
+      <c r="S4" s="88"/>
     </row>
     <row r="5" spans="1:19">
       <c r="A5" s="2"/>
@@ -6105,7 +6105,7 @@
       <c r="P5" s="17"/>
       <c r="Q5" s="17"/>
       <c r="R5" s="17"/>
-      <c r="S5" s="74"/>
+      <c r="S5" s="88"/>
     </row>
     <row r="6" spans="1:19">
       <c r="A6" s="2"/>
@@ -6126,7 +6126,7 @@
       <c r="P6" s="17"/>
       <c r="Q6" s="17"/>
       <c r="R6" s="17"/>
-      <c r="S6" s="74"/>
+      <c r="S6" s="88"/>
     </row>
     <row r="7" spans="1:19">
       <c r="A7" s="2"/>
@@ -6147,7 +6147,7 @@
       <c r="P7" s="26"/>
       <c r="Q7" s="26"/>
       <c r="R7" s="26"/>
-      <c r="S7" s="74"/>
+      <c r="S7" s="88"/>
     </row>
     <row r="8" spans="1:19">
       <c r="A8" s="2"/>
@@ -6168,7 +6168,7 @@
       <c r="P8" s="26"/>
       <c r="Q8" s="26"/>
       <c r="R8" s="26"/>
-      <c r="S8" s="74"/>
+      <c r="S8" s="88"/>
     </row>
     <row r="9" spans="1:19">
       <c r="A9" s="2"/>
@@ -6843,61 +6843,61 @@
       <c r="R20" s="35"/>
       <c r="S20" s="49"/>
     </row>
-    <row r="21" spans="1:19" s="86" customFormat="1">
-      <c r="A21" s="79"/>
-      <c r="B21" s="80">
+    <row r="21" spans="1:19" s="76" customFormat="1">
+      <c r="A21" s="69"/>
+      <c r="B21" s="70">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="81" t="s">
+      <c r="C21" s="71" t="s">
         <v>25</v>
       </c>
-      <c r="D21" s="82" t="s">
+      <c r="D21" s="72" t="s">
         <v>92</v>
       </c>
-      <c r="E21" s="82" t="s">
+      <c r="E21" s="72" t="s">
         <v>93</v>
       </c>
-      <c r="F21" s="82" t="s">
+      <c r="F21" s="72" t="s">
         <v>88</v>
       </c>
-      <c r="G21" s="82" t="s">
+      <c r="G21" s="72" t="s">
         <v>94</v>
       </c>
-      <c r="H21" s="82" t="s">
+      <c r="H21" s="72" t="s">
         <v>30</v>
       </c>
-      <c r="I21" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J21" s="82" t="s">
+      <c r="I21" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J21" s="72" t="s">
         <v>95</v>
       </c>
-      <c r="K21" s="82" t="s">
+      <c r="K21" s="72" t="s">
         <v>96</v>
       </c>
-      <c r="L21" s="82">
+      <c r="L21" s="72">
         <v>1</v>
       </c>
-      <c r="M21" s="83">
+      <c r="M21" s="73">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="N21" s="82">
+      <c r="N21" s="72">
         <v>100</v>
       </c>
-      <c r="O21" s="84" t="s">
-        <v>34</v>
-      </c>
-      <c r="P21" s="85">
+      <c r="O21" s="74" t="s">
+        <v>34</v>
+      </c>
+      <c r="P21" s="75">
         <v>3.8999999999999998E-3</v>
       </c>
-      <c r="Q21" s="85">
+      <c r="Q21" s="75">
         <f t="shared" si="1"/>
         <v>0.38999999999999996</v>
       </c>
-      <c r="R21" s="82"/>
-      <c r="S21" s="82"/>
+      <c r="R21" s="72"/>
+      <c r="S21" s="72"/>
     </row>
     <row r="22" spans="1:19" s="1" customFormat="1">
       <c r="A22" s="32"/>
@@ -7347,60 +7347,60 @@
       <c r="R29" s="37"/>
       <c r="S29" s="37"/>
     </row>
-    <row r="30" spans="1:19" s="86" customFormat="1">
-      <c r="A30" s="79"/>
-      <c r="B30" s="87">
+    <row r="30" spans="1:19" s="76" customFormat="1">
+      <c r="A30" s="69"/>
+      <c r="B30" s="77">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="81" t="s">
+      <c r="C30" s="71" t="s">
         <v>124</v>
       </c>
-      <c r="D30" s="83" t="s">
+      <c r="D30" s="73" t="s">
         <v>142</v>
       </c>
-      <c r="E30" s="83" t="s">
+      <c r="E30" s="73" t="s">
         <v>143</v>
       </c>
-      <c r="F30" s="83" t="s">
+      <c r="F30" s="73" t="s">
         <v>144</v>
       </c>
-      <c r="G30" s="83" t="s">
+      <c r="G30" s="73" t="s">
         <v>145</v>
       </c>
-      <c r="H30" s="83" t="s">
+      <c r="H30" s="73" t="s">
         <v>146</v>
       </c>
-      <c r="I30" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J30" s="83" t="s">
+      <c r="I30" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J30" s="73" t="s">
         <v>147</v>
       </c>
-      <c r="K30" s="83" t="s">
-        <v>31</v>
-      </c>
-      <c r="L30" s="83">
+      <c r="K30" s="73" t="s">
+        <v>31</v>
+      </c>
+      <c r="L30" s="73">
         <v>1</v>
       </c>
-      <c r="M30" s="83">
+      <c r="M30" s="73">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="N30" s="83">
+      <c r="N30" s="73">
         <v>20</v>
       </c>
-      <c r="O30" s="88" t="s">
-        <v>34</v>
-      </c>
-      <c r="P30" s="89">
+      <c r="O30" s="78" t="s">
+        <v>34</v>
+      </c>
+      <c r="P30" s="79">
         <v>3.4200000000000001E-2</v>
       </c>
-      <c r="Q30" s="89">
+      <c r="Q30" s="79">
         <f t="shared" si="1"/>
         <v>0.68400000000000005</v>
       </c>
-      <c r="R30" s="83"/>
+      <c r="R30" s="73"/>
       <c r="S30" s="64"/>
     </row>
     <row r="31" spans="1:19" s="1" customFormat="1" ht="24">
@@ -7629,61 +7629,61 @@
       </c>
       <c r="S34" s="49"/>
     </row>
-    <row r="35" spans="1:19" s="86" customFormat="1">
-      <c r="A35" s="79"/>
-      <c r="B35" s="80">
+    <row r="35" spans="1:19" s="76" customFormat="1">
+      <c r="A35" s="69"/>
+      <c r="B35" s="70">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="90" t="s">
+      <c r="C35" s="80" t="s">
         <v>170</v>
       </c>
-      <c r="D35" s="82" t="s">
+      <c r="D35" s="72" t="s">
         <v>171</v>
       </c>
-      <c r="E35" s="82" t="s">
+      <c r="E35" s="72" t="s">
         <v>172</v>
       </c>
-      <c r="F35" s="82" t="s">
+      <c r="F35" s="72" t="s">
         <v>173</v>
       </c>
-      <c r="G35" s="82" t="s">
+      <c r="G35" s="72" t="s">
         <v>174</v>
       </c>
-      <c r="H35" s="82" t="s">
+      <c r="H35" s="72" t="s">
         <v>175</v>
       </c>
-      <c r="I35" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J35" s="82" t="s">
+      <c r="I35" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J35" s="72" t="s">
         <v>176</v>
       </c>
-      <c r="K35" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="L35" s="82">
+      <c r="K35" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="L35" s="72">
         <v>1</v>
       </c>
-      <c r="M35" s="83">
+      <c r="M35" s="73">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="N35" s="82">
+      <c r="N35" s="72">
         <v>15</v>
       </c>
-      <c r="O35" s="91" t="s">
-        <v>34</v>
-      </c>
-      <c r="P35" s="85">
+      <c r="O35" s="81" t="s">
+        <v>34</v>
+      </c>
+      <c r="P35" s="75">
         <v>0.2029</v>
       </c>
-      <c r="Q35" s="85">
+      <c r="Q35" s="75">
         <f t="shared" ref="Q35:Q42" si="3">P35*N35</f>
         <v>3.0434999999999999</v>
       </c>
-      <c r="R35" s="82"/>
-      <c r="S35" s="82"/>
+      <c r="R35" s="72"/>
+      <c r="S35" s="72"/>
     </row>
     <row r="36" spans="1:19" s="1" customFormat="1" ht="24">
       <c r="A36" s="32"/>
@@ -7741,173 +7741,173 @@
       <c r="R36" s="35"/>
       <c r="S36" s="49"/>
     </row>
-    <row r="37" spans="1:19" s="86" customFormat="1">
-      <c r="A37" s="79"/>
-      <c r="B37" s="80">
+    <row r="37" spans="1:19" s="76" customFormat="1">
+      <c r="A37" s="69"/>
+      <c r="B37" s="70">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C37" s="90" t="s">
+      <c r="C37" s="80" t="s">
         <v>183</v>
       </c>
-      <c r="D37" s="82" t="s">
+      <c r="D37" s="72" t="s">
         <v>184</v>
       </c>
-      <c r="E37" s="82" t="s">
+      <c r="E37" s="72" t="s">
         <v>185</v>
       </c>
-      <c r="F37" s="82" t="s">
+      <c r="F37" s="72" t="s">
         <v>186</v>
       </c>
-      <c r="G37" s="82">
+      <c r="G37" s="72">
         <v>8266292</v>
       </c>
-      <c r="H37" s="82" t="s">
+      <c r="H37" s="72" t="s">
         <v>187</v>
       </c>
-      <c r="I37" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J37" s="82" t="s">
+      <c r="I37" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J37" s="72" t="s">
         <v>188</v>
       </c>
-      <c r="K37" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="L37" s="82">
+      <c r="K37" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="L37" s="72">
         <v>1</v>
       </c>
-      <c r="M37" s="83">
+      <c r="M37" s="73">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="N37" s="82">
+      <c r="N37" s="72">
         <v>11</v>
       </c>
-      <c r="O37" s="91" t="s">
-        <v>34</v>
-      </c>
-      <c r="P37" s="85">
+      <c r="O37" s="81" t="s">
+        <v>34</v>
+      </c>
+      <c r="P37" s="75">
         <v>0.25319999999999998</v>
       </c>
-      <c r="Q37" s="85">
+      <c r="Q37" s="75">
         <f t="shared" si="3"/>
         <v>2.7851999999999997</v>
       </c>
-      <c r="R37" s="82"/>
-      <c r="S37" s="82"/>
-    </row>
-    <row r="38" spans="1:19" s="86" customFormat="1">
-      <c r="A38" s="79"/>
-      <c r="B38" s="87">
+      <c r="R37" s="72"/>
+      <c r="S37" s="72"/>
+    </row>
+    <row r="38" spans="1:19" s="76" customFormat="1">
+      <c r="A38" s="69"/>
+      <c r="B38" s="77">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="81" t="s">
+      <c r="C38" s="71" t="s">
         <v>189</v>
       </c>
-      <c r="D38" s="83" t="s">
+      <c r="D38" s="73" t="s">
         <v>190</v>
       </c>
-      <c r="E38" s="83" t="s">
+      <c r="E38" s="73" t="s">
         <v>191</v>
       </c>
-      <c r="F38" s="83" t="s">
+      <c r="F38" s="73" t="s">
         <v>192</v>
       </c>
-      <c r="G38" s="83" t="s">
+      <c r="G38" s="73" t="s">
         <v>193</v>
       </c>
-      <c r="H38" s="83" t="s">
+      <c r="H38" s="73" t="s">
         <v>59</v>
       </c>
-      <c r="I38" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J38" s="83" t="s">
+      <c r="I38" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J38" s="73" t="s">
         <v>194</v>
       </c>
-      <c r="K38" s="83" t="s">
+      <c r="K38" s="73" t="s">
         <v>195</v>
       </c>
-      <c r="L38" s="83">
+      <c r="L38" s="73">
         <v>1</v>
       </c>
-      <c r="M38" s="83">
+      <c r="M38" s="73">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="N38" s="83">
+      <c r="N38" s="73">
         <v>15</v>
       </c>
-      <c r="O38" s="88" t="s">
-        <v>34</v>
-      </c>
-      <c r="P38" s="89">
+      <c r="O38" s="78" t="s">
+        <v>34</v>
+      </c>
+      <c r="P38" s="79">
         <v>0.2006</v>
       </c>
-      <c r="Q38" s="89">
+      <c r="Q38" s="79">
         <f t="shared" si="3"/>
         <v>3.0089999999999999</v>
       </c>
-      <c r="R38" s="83"/>
+      <c r="R38" s="73"/>
       <c r="S38" s="64"/>
     </row>
-    <row r="39" spans="1:19" s="86" customFormat="1">
-      <c r="A39" s="79"/>
-      <c r="B39" s="80">
+    <row r="39" spans="1:19" s="76" customFormat="1">
+      <c r="A39" s="69"/>
+      <c r="B39" s="70">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C39" s="90" t="s">
+      <c r="C39" s="80" t="s">
         <v>189</v>
       </c>
-      <c r="D39" s="82" t="s">
+      <c r="D39" s="72" t="s">
         <v>196</v>
       </c>
-      <c r="E39" s="82" t="s">
+      <c r="E39" s="72" t="s">
         <v>197</v>
       </c>
-      <c r="F39" s="82" t="s">
+      <c r="F39" s="72" t="s">
         <v>173</v>
       </c>
-      <c r="G39" s="82" t="s">
+      <c r="G39" s="72" t="s">
         <v>198</v>
       </c>
-      <c r="H39" s="82" t="s">
+      <c r="H39" s="72" t="s">
         <v>199</v>
       </c>
-      <c r="I39" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J39" s="82" t="s">
+      <c r="I39" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J39" s="72" t="s">
         <v>200</v>
       </c>
-      <c r="K39" s="82" t="s">
+      <c r="K39" s="72" t="s">
         <v>201</v>
       </c>
-      <c r="L39" s="82">
+      <c r="L39" s="72">
         <v>1</v>
       </c>
-      <c r="M39" s="83">
+      <c r="M39" s="73">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="N39" s="82">
+      <c r="N39" s="72">
         <v>20</v>
       </c>
-      <c r="O39" s="91" t="s">
-        <v>34</v>
-      </c>
-      <c r="P39" s="85">
+      <c r="O39" s="81" t="s">
+        <v>34</v>
+      </c>
+      <c r="P39" s="75">
         <v>6.6799999999999998E-2</v>
       </c>
-      <c r="Q39" s="85">
+      <c r="Q39" s="75">
         <f t="shared" si="3"/>
         <v>1.3359999999999999</v>
       </c>
-      <c r="R39" s="82"/>
-      <c r="S39" s="82"/>
+      <c r="R39" s="72"/>
+      <c r="S39" s="72"/>
     </row>
     <row r="40" spans="1:19" s="1" customFormat="1" ht="36">
       <c r="A40" s="32"/>
@@ -8021,7 +8021,7 @@
       <c r="R41" s="37"/>
       <c r="S41" s="37"/>
     </row>
-    <row r="42" spans="1:19" s="1" customFormat="1" ht="60">
+    <row r="42" spans="1:19" s="1" customFormat="1" ht="48">
       <c r="A42" s="32"/>
       <c r="B42" s="33">
         <f t="shared" si="0"/>
@@ -8188,7 +8188,7 @@
       <c r="R44" s="35"/>
       <c r="S44" s="49"/>
     </row>
-    <row r="45" spans="1:19" s="1" customFormat="1" ht="60">
+    <row r="45" spans="1:19" s="1" customFormat="1" ht="48">
       <c r="A45" s="32"/>
       <c r="B45" s="36">
         <f t="shared" si="0"/>
@@ -8300,116 +8300,116 @@
       <c r="R46" s="35"/>
       <c r="S46" s="49"/>
     </row>
-    <row r="47" spans="1:19" s="86" customFormat="1">
-      <c r="A47" s="79"/>
-      <c r="B47" s="80">
+    <row r="47" spans="1:19" s="76" customFormat="1">
+      <c r="A47" s="69"/>
+      <c r="B47" s="70">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C47" s="90" t="s">
+      <c r="C47" s="80" t="s">
         <v>237</v>
       </c>
-      <c r="D47" s="82" t="s">
+      <c r="D47" s="72" t="s">
         <v>244</v>
       </c>
-      <c r="E47" s="82" t="s">
+      <c r="E47" s="72" t="s">
         <v>245</v>
       </c>
-      <c r="F47" s="82" t="s">
+      <c r="F47" s="72" t="s">
         <v>246</v>
       </c>
-      <c r="G47" s="82" t="s">
+      <c r="G47" s="72" t="s">
         <v>247</v>
       </c>
-      <c r="H47" s="82" t="s">
+      <c r="H47" s="72" t="s">
         <v>30</v>
       </c>
-      <c r="I47" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J47" s="82" t="s">
+      <c r="I47" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J47" s="72" t="s">
         <v>248</v>
       </c>
-      <c r="K47" s="82" t="s">
+      <c r="K47" s="72" t="s">
         <v>249</v>
       </c>
-      <c r="L47" s="82">
+      <c r="L47" s="72">
         <v>2</v>
       </c>
-      <c r="M47" s="83">
+      <c r="M47" s="73">
         <f t="shared" si="4"/>
         <v>20</v>
       </c>
-      <c r="N47" s="82">
+      <c r="N47" s="72">
         <v>40</v>
       </c>
-      <c r="O47" s="91" t="s">
-        <v>34</v>
-      </c>
-      <c r="P47" s="85">
+      <c r="O47" s="81" t="s">
+        <v>34</v>
+      </c>
+      <c r="P47" s="75">
         <v>2.1700000000000001E-2</v>
       </c>
-      <c r="Q47" s="85">
+      <c r="Q47" s="75">
         <f t="shared" si="5"/>
         <v>0.86799999999999999</v>
       </c>
-      <c r="R47" s="82"/>
-      <c r="S47" s="82"/>
-    </row>
-    <row r="48" spans="1:19" s="86" customFormat="1">
-      <c r="A48" s="79"/>
-      <c r="B48" s="87">
+      <c r="R47" s="72"/>
+      <c r="S47" s="72"/>
+    </row>
+    <row r="48" spans="1:19" s="76" customFormat="1">
+      <c r="A48" s="69"/>
+      <c r="B48" s="77">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="C48" s="90" t="s">
+      <c r="C48" s="80" t="s">
         <v>237</v>
       </c>
-      <c r="D48" s="83" t="s">
+      <c r="D48" s="73" t="s">
         <v>250</v>
       </c>
-      <c r="E48" s="83" t="s">
+      <c r="E48" s="73" t="s">
         <v>251</v>
       </c>
-      <c r="F48" s="83" t="s">
+      <c r="F48" s="73" t="s">
         <v>252</v>
       </c>
-      <c r="G48" s="83" t="s">
+      <c r="G48" s="73" t="s">
         <v>253</v>
       </c>
-      <c r="H48" s="83" t="s">
+      <c r="H48" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="I48" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J48" s="83" t="s">
+      <c r="I48" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J48" s="73" t="s">
         <v>254</v>
       </c>
-      <c r="K48" s="83" t="s">
+      <c r="K48" s="73" t="s">
         <v>255</v>
       </c>
-      <c r="L48" s="83">
+      <c r="L48" s="73">
         <v>5</v>
       </c>
-      <c r="M48" s="83">
+      <c r="M48" s="73">
         <f t="shared" si="4"/>
         <v>50</v>
       </c>
-      <c r="N48" s="83">
+      <c r="N48" s="73">
         <v>60</v>
       </c>
-      <c r="O48" s="88" t="s">
-        <v>34</v>
-      </c>
-      <c r="P48" s="89">
+      <c r="O48" s="78" t="s">
+        <v>34</v>
+      </c>
+      <c r="P48" s="79">
         <v>1.41E-2</v>
       </c>
-      <c r="Q48" s="89">
+      <c r="Q48" s="79">
         <f t="shared" si="5"/>
         <v>0.84599999999999997</v>
       </c>
-      <c r="R48" s="83"/>
+      <c r="R48" s="73"/>
       <c r="S48" s="64"/>
     </row>
     <row r="49" spans="1:19" s="1" customFormat="1">
@@ -8524,61 +8524,61 @@
       <c r="R50" s="35"/>
       <c r="S50" s="49"/>
     </row>
-    <row r="51" spans="1:19" s="86" customFormat="1">
-      <c r="A51" s="79"/>
-      <c r="B51" s="80">
+    <row r="51" spans="1:19" s="76" customFormat="1">
+      <c r="A51" s="69"/>
+      <c r="B51" s="70">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="C51" s="90" t="s">
+      <c r="C51" s="80" t="s">
         <v>237</v>
       </c>
-      <c r="D51" s="82" t="s">
+      <c r="D51" s="72" t="s">
         <v>266</v>
       </c>
-      <c r="E51" s="82" t="s">
+      <c r="E51" s="72" t="s">
         <v>267</v>
       </c>
-      <c r="F51" s="82" t="s">
+      <c r="F51" s="72" t="s">
         <v>246</v>
       </c>
-      <c r="G51" s="82" t="s">
+      <c r="G51" s="72" t="s">
         <v>268</v>
       </c>
-      <c r="H51" s="82" t="s">
+      <c r="H51" s="72" t="s">
         <v>30</v>
       </c>
-      <c r="I51" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J51" s="82" t="s">
+      <c r="I51" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J51" s="72" t="s">
         <v>269</v>
       </c>
-      <c r="K51" s="82" t="s">
+      <c r="K51" s="72" t="s">
         <v>270</v>
       </c>
-      <c r="L51" s="82">
+      <c r="L51" s="72">
         <v>3</v>
       </c>
-      <c r="M51" s="83">
+      <c r="M51" s="73">
         <f t="shared" si="4"/>
         <v>30</v>
       </c>
-      <c r="N51" s="82">
+      <c r="N51" s="72">
         <v>100</v>
       </c>
-      <c r="O51" s="84" t="s">
-        <v>34</v>
-      </c>
-      <c r="P51" s="85">
+      <c r="O51" s="74" t="s">
+        <v>34</v>
+      </c>
+      <c r="P51" s="75">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="Q51" s="85">
+      <c r="Q51" s="75">
         <f t="shared" si="5"/>
         <v>0.11</v>
       </c>
-      <c r="R51" s="82"/>
-      <c r="S51" s="82"/>
+      <c r="R51" s="72"/>
+      <c r="S51" s="72"/>
     </row>
     <row r="52" spans="1:19" s="1" customFormat="1" ht="36">
       <c r="A52" s="32"/>
@@ -8692,172 +8692,172 @@
       <c r="R53" s="37"/>
       <c r="S53" s="37"/>
     </row>
-    <row r="54" spans="1:19" s="86" customFormat="1">
-      <c r="A54" s="79"/>
-      <c r="B54" s="87">
+    <row r="54" spans="1:19" s="76" customFormat="1">
+      <c r="A54" s="69"/>
+      <c r="B54" s="77">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="C54" s="81" t="s">
+      <c r="C54" s="71" t="s">
         <v>237</v>
       </c>
-      <c r="D54" s="83" t="s">
+      <c r="D54" s="73" t="s">
         <v>283</v>
       </c>
-      <c r="E54" s="83" t="s">
+      <c r="E54" s="73" t="s">
         <v>284</v>
       </c>
-      <c r="F54" s="83" t="s">
+      <c r="F54" s="73" t="s">
         <v>246</v>
       </c>
-      <c r="G54" s="83" t="s">
+      <c r="G54" s="73" t="s">
         <v>285</v>
       </c>
-      <c r="H54" s="83" t="s">
+      <c r="H54" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="I54" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J54" s="83" t="s">
+      <c r="I54" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J54" s="73" t="s">
         <v>286</v>
       </c>
-      <c r="K54" s="83" t="s">
+      <c r="K54" s="73" t="s">
         <v>287</v>
       </c>
-      <c r="L54" s="83">
+      <c r="L54" s="73">
         <v>1</v>
       </c>
-      <c r="M54" s="83">
+      <c r="M54" s="73">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="N54" s="83">
+      <c r="N54" s="73">
         <v>100</v>
       </c>
-      <c r="O54" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="P54" s="89">
+      <c r="O54" s="82" t="s">
+        <v>34</v>
+      </c>
+      <c r="P54" s="79">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="Q54" s="89">
+      <c r="Q54" s="79">
         <f t="shared" si="5"/>
         <v>0.21</v>
       </c>
-      <c r="R54" s="83"/>
+      <c r="R54" s="73"/>
       <c r="S54" s="64"/>
     </row>
-    <row r="55" spans="1:19" s="86" customFormat="1">
-      <c r="A55" s="79"/>
-      <c r="B55" s="80">
+    <row r="55" spans="1:19" s="76" customFormat="1">
+      <c r="A55" s="69"/>
+      <c r="B55" s="70">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="C55" s="81" t="s">
+      <c r="C55" s="71" t="s">
         <v>237</v>
       </c>
-      <c r="D55" s="82" t="s">
+      <c r="D55" s="72" t="s">
         <v>288</v>
       </c>
-      <c r="E55" s="82" t="s">
+      <c r="E55" s="72" t="s">
         <v>289</v>
       </c>
-      <c r="F55" s="82" t="s">
+      <c r="F55" s="72" t="s">
         <v>246</v>
       </c>
-      <c r="G55" s="82" t="s">
+      <c r="G55" s="72" t="s">
         <v>290</v>
       </c>
-      <c r="H55" s="82" t="s">
+      <c r="H55" s="72" t="s">
         <v>30</v>
       </c>
-      <c r="I55" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J55" s="82" t="s">
+      <c r="I55" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J55" s="72" t="s">
         <v>291</v>
       </c>
-      <c r="K55" s="82" t="s">
+      <c r="K55" s="72" t="s">
         <v>292</v>
       </c>
-      <c r="L55" s="82">
+      <c r="L55" s="72">
         <v>1</v>
       </c>
-      <c r="M55" s="83">
+      <c r="M55" s="73">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="N55" s="82">
+      <c r="N55" s="72">
         <v>20</v>
       </c>
-      <c r="O55" s="84" t="s">
-        <v>34</v>
-      </c>
-      <c r="P55" s="85">
+      <c r="O55" s="74" t="s">
+        <v>34</v>
+      </c>
+      <c r="P55" s="75">
         <v>3.7499999999999999E-2</v>
       </c>
-      <c r="Q55" s="85">
+      <c r="Q55" s="75">
         <f t="shared" si="5"/>
         <v>0.75</v>
       </c>
-      <c r="R55" s="82"/>
-      <c r="S55" s="82"/>
-    </row>
-    <row r="56" spans="1:19" s="86" customFormat="1">
-      <c r="A56" s="79"/>
-      <c r="B56" s="87">
+      <c r="R55" s="72"/>
+      <c r="S55" s="72"/>
+    </row>
+    <row r="56" spans="1:19" s="76" customFormat="1">
+      <c r="A56" s="69"/>
+      <c r="B56" s="77">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
-      <c r="C56" s="81" t="s">
+      <c r="C56" s="71" t="s">
         <v>293</v>
       </c>
-      <c r="D56" s="83" t="s">
+      <c r="D56" s="73" t="s">
         <v>294</v>
       </c>
-      <c r="E56" s="83" t="s">
+      <c r="E56" s="73" t="s">
         <v>295</v>
       </c>
-      <c r="F56" s="83" t="s">
+      <c r="F56" s="73" t="s">
         <v>296</v>
       </c>
-      <c r="G56" s="83" t="s">
+      <c r="G56" s="73" t="s">
         <v>296</v>
       </c>
-      <c r="H56" s="83" t="s">
+      <c r="H56" s="73" t="s">
         <v>297</v>
       </c>
-      <c r="I56" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J56" s="83" t="s">
+      <c r="I56" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J56" s="73" t="s">
         <v>298</v>
       </c>
-      <c r="K56" s="83" t="s">
-        <v>31</v>
-      </c>
-      <c r="L56" s="83">
+      <c r="K56" s="73" t="s">
+        <v>31</v>
+      </c>
+      <c r="L56" s="73">
         <v>2</v>
       </c>
-      <c r="M56" s="83">
+      <c r="M56" s="73">
         <f t="shared" si="4"/>
         <v>20</v>
       </c>
-      <c r="N56" s="83">
+      <c r="N56" s="73">
         <v>25</v>
       </c>
-      <c r="O56" s="88" t="s">
-        <v>34</v>
-      </c>
-      <c r="P56" s="89">
+      <c r="O56" s="78" t="s">
+        <v>34</v>
+      </c>
+      <c r="P56" s="79">
         <v>0.1729</v>
       </c>
-      <c r="Q56" s="89">
+      <c r="Q56" s="79">
         <f t="shared" si="5"/>
         <v>4.3224999999999998</v>
       </c>
-      <c r="R56" s="83"/>
+      <c r="R56" s="73"/>
       <c r="S56" s="64"/>
     </row>
     <row r="57" spans="1:19" s="1" customFormat="1">
@@ -8907,69 +8907,69 @@
         <v>316</v>
       </c>
       <c r="P57" s="44">
-        <v>8.3000000000000007</v>
+        <v>16.25</v>
       </c>
       <c r="Q57" s="44">
         <f t="shared" si="5"/>
-        <v>91.300000000000011</v>
+        <v>178.75</v>
       </c>
       <c r="R57" s="37"/>
       <c r="S57" s="37"/>
     </row>
-    <row r="58" spans="1:19" s="86" customFormat="1">
-      <c r="A58" s="79"/>
-      <c r="B58" s="87">
+    <row r="58" spans="1:19" s="76" customFormat="1">
+      <c r="A58" s="69"/>
+      <c r="B58" s="77">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-      <c r="C58" s="81" t="s">
+      <c r="C58" s="71" t="s">
         <v>299</v>
       </c>
-      <c r="D58" s="83" t="s">
+      <c r="D58" s="73" t="s">
         <v>305</v>
       </c>
-      <c r="E58" s="83" t="s">
+      <c r="E58" s="73" t="s">
         <v>306</v>
       </c>
-      <c r="F58" s="83" t="s">
+      <c r="F58" s="73" t="s">
         <v>307</v>
       </c>
-      <c r="G58" s="83" t="s">
+      <c r="G58" s="73" t="s">
         <v>308</v>
       </c>
-      <c r="H58" s="83" t="s">
+      <c r="H58" s="73" t="s">
         <v>309</v>
       </c>
-      <c r="I58" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J58" s="83" t="s">
+      <c r="I58" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J58" s="73" t="s">
         <v>310</v>
       </c>
-      <c r="K58" s="83" t="s">
-        <v>31</v>
-      </c>
-      <c r="L58" s="83">
+      <c r="K58" s="73" t="s">
+        <v>31</v>
+      </c>
+      <c r="L58" s="73">
         <v>1</v>
       </c>
-      <c r="M58" s="83">
+      <c r="M58" s="73">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="N58" s="83">
+      <c r="N58" s="73">
         <v>11</v>
       </c>
-      <c r="O58" s="88" t="s">
-        <v>34</v>
-      </c>
-      <c r="P58" s="89">
+      <c r="O58" s="78" t="s">
+        <v>34</v>
+      </c>
+      <c r="P58" s="79">
         <v>0.66659999999999997</v>
       </c>
-      <c r="Q58" s="89">
+      <c r="Q58" s="79">
         <f t="shared" si="5"/>
         <v>7.3325999999999993</v>
       </c>
-      <c r="R58" s="83"/>
+      <c r="R58" s="73"/>
       <c r="S58" s="64"/>
     </row>
     <row r="59" spans="1:19" s="1" customFormat="1">
@@ -9246,58 +9246,58 @@
       <c r="R63" s="37"/>
       <c r="S63" s="37"/>
     </row>
-    <row r="64" spans="1:19" s="86" customFormat="1">
-      <c r="A64" s="79"/>
-      <c r="B64" s="87">
+    <row r="64" spans="1:19" s="76" customFormat="1">
+      <c r="A64" s="69"/>
+      <c r="B64" s="77">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
-      <c r="C64" s="81" t="s">
+      <c r="C64" s="71" t="s">
         <v>299</v>
       </c>
-      <c r="D64" s="83" t="s">
+      <c r="D64" s="73" t="s">
         <v>341</v>
       </c>
-      <c r="E64" s="83" t="s">
+      <c r="E64" s="73" t="s">
         <v>342</v>
       </c>
-      <c r="F64" s="83" t="s">
+      <c r="F64" s="73" t="s">
         <v>343</v>
       </c>
-      <c r="G64" s="83" t="s">
+      <c r="G64" s="73" t="s">
         <v>344</v>
       </c>
-      <c r="H64" s="83" t="s">
+      <c r="H64" s="73" t="s">
         <v>327</v>
       </c>
-      <c r="I64" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J64" s="83" t="s">
+      <c r="I64" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J64" s="73" t="s">
         <v>345</v>
       </c>
-      <c r="K64" s="83"/>
-      <c r="L64" s="83">
+      <c r="K64" s="73"/>
+      <c r="L64" s="73">
         <v>1</v>
       </c>
-      <c r="M64" s="83">
+      <c r="M64" s="73">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="N64" s="83">
+      <c r="N64" s="73">
         <v>11</v>
       </c>
-      <c r="O64" s="88" t="s">
-        <v>34</v>
-      </c>
-      <c r="P64" s="89">
+      <c r="O64" s="78" t="s">
+        <v>34</v>
+      </c>
+      <c r="P64" s="79">
         <v>0.96409999999999996</v>
       </c>
-      <c r="Q64" s="89">
+      <c r="Q64" s="79">
         <f t="shared" si="5"/>
         <v>10.6051</v>
       </c>
-      <c r="R64" s="83"/>
+      <c r="R64" s="73"/>
       <c r="S64" s="64"/>
     </row>
     <row r="65" spans="1:19" s="1" customFormat="1" ht="36">
@@ -9356,60 +9356,60 @@
       <c r="R65" s="37"/>
       <c r="S65" s="37"/>
     </row>
-    <row r="66" spans="1:19" s="86" customFormat="1">
-      <c r="A66" s="79"/>
-      <c r="B66" s="87">
+    <row r="66" spans="1:19" s="76" customFormat="1">
+      <c r="A66" s="69"/>
+      <c r="B66" s="77">
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
-      <c r="C66" s="90" t="s">
+      <c r="C66" s="80" t="s">
         <v>346</v>
       </c>
-      <c r="D66" s="83" t="s">
+      <c r="D66" s="73" t="s">
         <v>353</v>
       </c>
-      <c r="E66" s="83" t="s">
+      <c r="E66" s="73" t="s">
         <v>354</v>
       </c>
-      <c r="F66" s="82" t="s">
+      <c r="F66" s="72" t="s">
         <v>173</v>
       </c>
-      <c r="G66" s="83" t="s">
+      <c r="G66" s="73" t="s">
         <v>355</v>
       </c>
-      <c r="H66" s="83" t="s">
+      <c r="H66" s="73" t="s">
         <v>356</v>
       </c>
-      <c r="I66" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="J66" s="83" t="s">
+      <c r="I66" s="72" t="s">
+        <v>31</v>
+      </c>
+      <c r="J66" s="73" t="s">
         <v>357</v>
       </c>
-      <c r="K66" s="83" t="s">
+      <c r="K66" s="73" t="s">
         <v>358</v>
       </c>
-      <c r="L66" s="83">
+      <c r="L66" s="73">
         <v>1</v>
       </c>
-      <c r="M66" s="83">
+      <c r="M66" s="73">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="N66" s="83">
+      <c r="N66" s="73">
         <v>15</v>
       </c>
-      <c r="O66" s="88" t="s">
-        <v>34</v>
-      </c>
-      <c r="P66" s="89">
+      <c r="O66" s="78" t="s">
+        <v>34</v>
+      </c>
+      <c r="P66" s="79">
         <v>0.1401</v>
       </c>
-      <c r="Q66" s="89">
+      <c r="Q66" s="79">
         <f t="shared" si="5"/>
         <v>2.1015000000000001</v>
       </c>
-      <c r="R66" s="83"/>
+      <c r="R66" s="73"/>
       <c r="S66" s="64"/>
     </row>
     <row r="67" spans="1:19">
@@ -9569,17 +9569,17 @@
       <c r="K70" s="56"/>
       <c r="L70" s="56"/>
       <c r="M70" s="56"/>
-      <c r="N70" s="71" t="s">
+      <c r="N70" s="85" t="s">
         <v>359</v>
       </c>
-      <c r="O70" s="72"/>
-      <c r="P70" s="72"/>
+      <c r="O70" s="86"/>
+      <c r="P70" s="86"/>
       <c r="Q70" s="61">
         <f>SUM(Q10:Q69)</f>
-        <v>648.11609999999996</v>
-      </c>
-      <c r="R70" s="75"/>
-      <c r="S70" s="76"/>
+        <v>735.56609999999989</v>
+      </c>
+      <c r="R70" s="89"/>
+      <c r="S70" s="90"/>
     </row>
     <row r="71" spans="1:19" ht="18.75">
       <c r="A71" s="2"/>
@@ -9595,17 +9595,17 @@
       <c r="K71" s="60"/>
       <c r="L71" s="60"/>
       <c r="M71" s="60"/>
-      <c r="N71" s="71" t="s">
+      <c r="N71" s="85" t="s">
         <v>360</v>
       </c>
-      <c r="O71" s="72"/>
-      <c r="P71" s="72"/>
+      <c r="O71" s="86"/>
+      <c r="P71" s="86"/>
       <c r="Q71" s="62">
         <f>Q70/10</f>
-        <v>64.811610000000002</v>
-      </c>
-      <c r="R71" s="77"/>
-      <c r="S71" s="78"/>
+        <v>73.556609999999992</v>
+      </c>
+      <c r="R71" s="91"/>
+      <c r="S71" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>